<commit_message>
Crear usuarios y asignar roles
</commit_message>
<xml_diff>
--- a/RubricaPlitix.xlsx
+++ b/RubricaPlitix.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\jcalc\Documentos\Carrera\Cuarto\plytix-ABBDD\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B2FDA97D-2E46-43D9-AAE9-6898B37F0DA1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A3961D30-4C15-4581-9F3E-4BAF90047169}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11020" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="149" uniqueCount="101">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="153" uniqueCount="105">
   <si>
     <t>Miscelanea</t>
   </si>
@@ -357,6 +357,19 @@
   </si>
   <si>
     <t>Se audita la tabla PLAN: SELECT event_timestamp, dbusername, action_name, object_name, sql_text FROM UNIFIED_AUDIT_TRAIL WHERE object_name = 'PLAN' ORDER BY event_timestamp DESC;</t>
+  </si>
+  <si>
+    <t>Se asignan a través de los roles, solo tienen permiso para acceder a las vistas correspondientes que se han creado para este propósito en la entrega 2 de nivel físico</t>
+  </si>
+  <si>
+    <t>SELECT * FROM DBA_ROLES
+WHERE ROLE IN ('R_USER_STD', 'R_GESTOR_CUENTA', 'R_PLANIFICADOR_SERVICIOS');</t>
+  </si>
+  <si>
+    <t>El administrador del sistema es el propio PLYTIX. Se ha creado el usuario anagarcia como ejemplo de usuario estándar, el usuario gestorcuentas y el usuario planificador correspondiente a los otros dos roles</t>
+  </si>
+  <si>
+    <t>Las especificadas en el enunciado 2 de la parte de nivel físico, se otorgan mediante roles</t>
   </si>
 </sst>
 </file>
@@ -1465,7 +1478,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="33" spans="1:20" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="33" spans="1:20" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A33" s="19">
         <f>A32+1</f>
         <v>11</v>
@@ -1479,52 +1492,60 @@
       <c r="D33" s="13" t="s">
         <v>6</v>
       </c>
-      <c r="E33" s="12"/>
+      <c r="E33" s="12" t="s">
+        <v>102</v>
+      </c>
       <c r="F33">
         <f t="shared" ref="F33:F38" si="1">IF(D33="SI",1,0)</f>
         <v>1</v>
       </c>
     </row>
-    <row r="34" spans="1:20" x14ac:dyDescent="0.35">
+    <row r="34" spans="1:20" ht="58" x14ac:dyDescent="0.35">
       <c r="B34" s="5"/>
       <c r="C34" s="5" t="s">
         <v>21</v>
       </c>
       <c r="D34" s="13" t="s">
-        <v>7</v>
-      </c>
-      <c r="E34" s="12"/>
+        <v>6</v>
+      </c>
+      <c r="E34" s="12" t="s">
+        <v>103</v>
+      </c>
       <c r="F34">
         <f t="shared" si="1"/>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="35" spans="1:20" ht="29" x14ac:dyDescent="0.35">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="35" spans="1:20" ht="43.5" x14ac:dyDescent="0.35">
       <c r="B35" s="5"/>
       <c r="C35" s="5" t="s">
         <v>22</v>
       </c>
       <c r="D35" s="13" t="s">
-        <v>7</v>
-      </c>
-      <c r="E35" s="12"/>
+        <v>6</v>
+      </c>
+      <c r="E35" s="12" t="s">
+        <v>101</v>
+      </c>
       <c r="F35">
         <f t="shared" si="1"/>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="36" spans="1:20" x14ac:dyDescent="0.35">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="36" spans="1:20" ht="29" x14ac:dyDescent="0.35">
       <c r="B36" s="5"/>
       <c r="C36" s="5" t="s">
         <v>42</v>
       </c>
       <c r="D36" s="13" t="s">
-        <v>7</v>
-      </c>
-      <c r="E36" s="12"/>
+        <v>6</v>
+      </c>
+      <c r="E36" s="12" t="s">
+        <v>104</v>
+      </c>
       <c r="F36">
         <f t="shared" si="1"/>
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="37" spans="1:20" ht="101.5" x14ac:dyDescent="0.35">
@@ -1566,7 +1587,7 @@
       <c r="E39" s="9"/>
       <c r="F39" s="11">
         <f>SUM(F6:F38)/COUNT(F6:F38)*2</f>
-        <v>1.7575757575757576</v>
+        <v>1.9393939393939394</v>
       </c>
     </row>
     <row r="40" spans="1:20" ht="23.5" x14ac:dyDescent="0.55000000000000004">
@@ -1878,7 +1899,7 @@
       <c r="C60" s="5"/>
       <c r="F60" s="10">
         <f>F59+F39</f>
-        <v>3.1861471861471862</v>
+        <v>3.3679653679653683</v>
       </c>
       <c r="G60" s="10"/>
       <c r="H60" s="10"/>

</xml_diff>

<commit_message>
Confirmado/deshecho las transacciones en los procedimientos
</commit_message>
<xml_diff>
--- a/RubricaPlitix.xlsx
+++ b/RubricaPlitix.xlsx
@@ -5,12 +5,12 @@
   <workbookPr autoCompressPictures="0"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\jcalc\Documentos\Carrera\Cuarto\plytix-ABBDD\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\pablo\Desktop\abbddef\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A3961D30-4C15-4581-9F3E-4BAF90047169}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9115CA56-CD2F-4D54-A46E-BEE20791B452}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11020" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="11424" yWindow="0" windowWidth="11712" windowHeight="12336" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Hoja1" sheetId="3" r:id="rId1"/>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="153" uniqueCount="105">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="154" uniqueCount="106">
   <si>
     <t>Miscelanea</t>
   </si>
@@ -370,6 +370,9 @@
   </si>
   <si>
     <t>Las especificadas en el enunciado 2 de la parte de nivel físico, se otorgan mediante roles</t>
+  </si>
+  <si>
+    <t>Sí, en los procedimientos contenidos en los paquetes, las transacciones se confirman (COMMIT) tras completarse correctamente o después de insertar en la tabla TRAZA en caso de que ocurra una excepción. En los casos en los que no es necesario emplear dicha tabla, los cambios se revierten (ROLLBACK) para mantener la integridad de los datos.</t>
   </si>
 </sst>
 </file>
@@ -939,16 +942,16 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5C334588-D4EB-43EC-8424-5ED08F8B2503}">
   <dimension ref="A1:U61"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="12" customWidth="1"/>
-    <col min="2" max="2" width="51.1796875" customWidth="1"/>
-    <col min="3" max="3" width="46.1796875" customWidth="1"/>
-    <col min="5" max="5" width="47.7265625" style="5" customWidth="1"/>
-    <col min="6" max="8" width="11.453125" customWidth="1"/>
+    <col min="2" max="2" width="51.21875" customWidth="1"/>
+    <col min="3" max="3" width="46.21875" customWidth="1"/>
+    <col min="5" max="5" width="47.77734375" style="5" customWidth="1"/>
+    <col min="6" max="8" width="11.44140625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:21" ht="23.5" x14ac:dyDescent="0.55000000000000004">
+    <row r="1" spans="1:21" ht="23.4" x14ac:dyDescent="0.45">
       <c r="A1" s="7"/>
       <c r="B1" s="7" t="s">
         <v>4</v>
@@ -958,7 +961,7 @@
       <c r="E1" s="8"/>
       <c r="F1" s="7"/>
     </row>
-    <row r="2" spans="1:21" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:21" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A2" s="17" t="s">
         <v>35</v>
       </c>
@@ -968,7 +971,7 @@
       <c r="E2" s="15"/>
       <c r="F2" s="14"/>
     </row>
-    <row r="3" spans="1:21" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A3" s="1"/>
       <c r="B3" s="2"/>
       <c r="C3" s="2"/>
@@ -978,7 +981,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="4" spans="1:21" ht="29" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:21" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A4" s="3" t="s">
         <v>3</v>
       </c>
@@ -1009,14 +1012,14 @@
       <c r="T4" s="3"/>
       <c r="U4" s="3"/>
     </row>
-    <row r="5" spans="1:21" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:21" ht="15.6" x14ac:dyDescent="0.3">
       <c r="B5" s="18" t="s">
         <v>28</v>
       </c>
       <c r="C5" s="4"/>
       <c r="D5" s="4"/>
     </row>
-    <row r="6" spans="1:21" ht="29" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:21" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A6" s="19">
         <v>1</v>
       </c>
@@ -1037,7 +1040,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="7" spans="1:21" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:21" ht="43.2" x14ac:dyDescent="0.3">
       <c r="B7" s="5"/>
       <c r="C7" s="5" t="s">
         <v>13</v>
@@ -1053,7 +1056,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="8" spans="1:21" ht="58" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:21" ht="57.6" x14ac:dyDescent="0.3">
       <c r="B8" s="5"/>
       <c r="C8" s="5" t="s">
         <v>49</v>
@@ -1069,7 +1072,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="9" spans="1:21" ht="87" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:21" ht="86.4" x14ac:dyDescent="0.3">
       <c r="B9" s="5"/>
       <c r="C9" s="5" t="s">
         <v>69</v>
@@ -1085,7 +1088,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="10" spans="1:21" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:21" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A10" s="19">
         <f>A6+1</f>
         <v>2</v>
@@ -1107,7 +1110,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="11" spans="1:21" ht="72.5" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:21" ht="72" x14ac:dyDescent="0.3">
       <c r="B11" s="5"/>
       <c r="C11" s="5" t="s">
         <v>41</v>
@@ -1123,7 +1126,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="12" spans="1:21" ht="58" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:21" ht="57.6" x14ac:dyDescent="0.3">
       <c r="A12" s="19">
         <f>A10+1</f>
         <v>3</v>
@@ -1145,7 +1148,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="13" spans="1:21" ht="29" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:21" ht="28.8" x14ac:dyDescent="0.3">
       <c r="B13" s="5"/>
       <c r="C13" s="5" t="s">
         <v>76</v>
@@ -1161,7 +1164,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="14" spans="1:21" ht="72.5" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:21" ht="72" x14ac:dyDescent="0.3">
       <c r="A14" s="19">
         <v>4</v>
       </c>
@@ -1182,7 +1185,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="15" spans="1:21" ht="72.5" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:21" ht="72" x14ac:dyDescent="0.3">
       <c r="C15" s="21" t="s">
         <v>51</v>
       </c>
@@ -1197,7 +1200,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="16" spans="1:21" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:21" ht="43.2" x14ac:dyDescent="0.3">
       <c r="B16" s="5"/>
       <c r="C16" s="21" t="s">
         <v>52</v>
@@ -1213,7 +1216,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="17" spans="1:6" ht="72.5" x14ac:dyDescent="0.35">
+    <row r="17" spans="1:6" ht="72" x14ac:dyDescent="0.3">
       <c r="B17" s="5"/>
       <c r="C17" s="21" t="s">
         <v>53</v>
@@ -1229,7 +1232,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="18" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="18" spans="1:6" x14ac:dyDescent="0.3">
       <c r="B18" s="5"/>
       <c r="C18" s="21" t="s">
         <v>54</v>
@@ -1245,7 +1248,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="19" spans="1:6" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="19" spans="1:6" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A19" s="19">
         <v>5</v>
       </c>
@@ -1266,7 +1269,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="20" spans="1:6" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="20" spans="1:6" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A20" s="19">
         <f>A19+1</f>
         <v>6</v>
@@ -1286,7 +1289,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="21" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="21" spans="1:6" x14ac:dyDescent="0.3">
       <c r="B21" s="5"/>
       <c r="C21" s="22" t="s">
         <v>57</v>
@@ -1300,7 +1303,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="22" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="22" spans="1:6" x14ac:dyDescent="0.3">
       <c r="B22" s="23"/>
       <c r="C22" s="22" t="s">
         <v>58</v>
@@ -1314,7 +1317,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="23" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="23" spans="1:6" x14ac:dyDescent="0.3">
       <c r="B23" s="23"/>
       <c r="C23" s="22" t="s">
         <v>70</v>
@@ -1328,7 +1331,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="24" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="24" spans="1:6" x14ac:dyDescent="0.3">
       <c r="B24" s="23"/>
       <c r="C24" s="24" t="s">
         <v>59</v>
@@ -1342,7 +1345,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="25" spans="1:6" ht="25.9" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="25" spans="1:6" ht="25.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B25" s="23"/>
       <c r="C25" s="22" t="s">
         <v>60</v>
@@ -1356,7 +1359,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="26" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="26" spans="1:6" x14ac:dyDescent="0.3">
       <c r="C26" s="22" t="s">
         <v>61</v>
       </c>
@@ -1368,7 +1371,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="27" spans="1:6" ht="25.9" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="27" spans="1:6" ht="25.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B27" s="23"/>
       <c r="C27" s="22" t="s">
         <v>62</v>
@@ -1382,7 +1385,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="28" spans="1:6" ht="25.9" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="28" spans="1:6" ht="25.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B28" s="23"/>
       <c r="C28" s="22" t="s">
         <v>71</v>
@@ -1396,7 +1399,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="29" spans="1:6" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="29" spans="1:6" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A29" s="19">
         <f>A20+1</f>
         <v>7</v>
@@ -1416,7 +1419,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="30" spans="1:6" ht="29" x14ac:dyDescent="0.35">
+    <row r="30" spans="1:6" ht="100.8" x14ac:dyDescent="0.3">
       <c r="A30" s="19">
         <f>A29+1</f>
         <v>8</v>
@@ -1428,15 +1431,17 @@
         <v>32</v>
       </c>
       <c r="D30" s="13" t="s">
-        <v>7</v>
-      </c>
-      <c r="E30" s="12"/>
+        <v>6</v>
+      </c>
+      <c r="E30" s="12" t="s">
+        <v>105</v>
+      </c>
       <c r="F30">
         <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="31" spans="1:6" ht="29" x14ac:dyDescent="0.35">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="31" spans="1:6" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A31" s="19">
         <f>A30+1</f>
         <v>9</v>
@@ -1458,7 +1463,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="32" spans="1:6" ht="29" x14ac:dyDescent="0.35">
+    <row r="32" spans="1:6" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A32" s="19">
         <f>A31+1</f>
         <v>10</v>
@@ -1478,7 +1483,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="33" spans="1:20" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="33" spans="1:20" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A33" s="19">
         <f>A32+1</f>
         <v>11</v>
@@ -1500,7 +1505,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="34" spans="1:20" ht="58" x14ac:dyDescent="0.35">
+    <row r="34" spans="1:20" ht="57.6" x14ac:dyDescent="0.3">
       <c r="B34" s="5"/>
       <c r="C34" s="5" t="s">
         <v>21</v>
@@ -1516,7 +1521,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="35" spans="1:20" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="35" spans="1:20" ht="43.2" x14ac:dyDescent="0.3">
       <c r="B35" s="5"/>
       <c r="C35" s="5" t="s">
         <v>22</v>
@@ -1532,7 +1537,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="36" spans="1:20" ht="29" x14ac:dyDescent="0.35">
+    <row r="36" spans="1:20" ht="28.8" x14ac:dyDescent="0.3">
       <c r="B36" s="5"/>
       <c r="C36" s="5" t="s">
         <v>42</v>
@@ -1548,7 +1553,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="37" spans="1:20" ht="101.5" x14ac:dyDescent="0.35">
+    <row r="37" spans="1:20" ht="100.8" x14ac:dyDescent="0.3">
       <c r="B37" s="5"/>
       <c r="C37" s="5" t="s">
         <v>23</v>
@@ -1564,7 +1569,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="38" spans="1:20" x14ac:dyDescent="0.35">
+    <row r="38" spans="1:20" x14ac:dyDescent="0.3">
       <c r="B38" s="5"/>
       <c r="C38" s="5" t="s">
         <v>33</v>
@@ -1580,17 +1585,17 @@
         <v>1</v>
       </c>
     </row>
-    <row r="39" spans="1:20" x14ac:dyDescent="0.35">
+    <row r="39" spans="1:20" x14ac:dyDescent="0.3">
       <c r="B39" s="5"/>
       <c r="C39" s="5"/>
       <c r="D39" s="5"/>
       <c r="E39" s="9"/>
       <c r="F39" s="11">
         <f>SUM(F6:F38)/COUNT(F6:F38)*2</f>
-        <v>1.9393939393939394</v>
-      </c>
-    </row>
-    <row r="40" spans="1:20" ht="23.5" x14ac:dyDescent="0.55000000000000004">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="40" spans="1:20" ht="23.4" x14ac:dyDescent="0.45">
       <c r="B40" s="25" t="s">
         <v>9</v>
       </c>
@@ -1612,7 +1617,7 @@
       <c r="S40" s="10"/>
       <c r="T40" s="10"/>
     </row>
-    <row r="41" spans="1:20" ht="23.5" x14ac:dyDescent="0.55000000000000004">
+    <row r="41" spans="1:20" ht="23.4" x14ac:dyDescent="0.45">
       <c r="B41" s="25" t="s">
         <v>10</v>
       </c>
@@ -1620,7 +1625,7 @@
       <c r="D41" s="5"/>
       <c r="E41" s="9"/>
     </row>
-    <row r="42" spans="1:20" ht="23.5" x14ac:dyDescent="0.55000000000000004">
+    <row r="42" spans="1:20" ht="23.4" x14ac:dyDescent="0.45">
       <c r="B42" s="25" t="s">
         <v>11</v>
       </c>
@@ -1628,17 +1633,17 @@
       <c r="D42" s="5"/>
       <c r="E42" s="9"/>
     </row>
-    <row r="43" spans="1:20" x14ac:dyDescent="0.35">
+    <row r="43" spans="1:20" x14ac:dyDescent="0.3">
       <c r="B43" s="5"/>
       <c r="C43" s="5"/>
       <c r="D43" s="5"/>
       <c r="E43" s="9"/>
     </row>
-    <row r="44" spans="1:20" x14ac:dyDescent="0.35">
+    <row r="44" spans="1:20" x14ac:dyDescent="0.3">
       <c r="B44" s="5"/>
       <c r="E44" s="9"/>
     </row>
-    <row r="45" spans="1:20" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="45" spans="1:20" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A45" s="19">
         <v>1</v>
       </c>
@@ -1659,7 +1664,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="46" spans="1:20" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="46" spans="1:20" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A46" s="17"/>
       <c r="B46" s="26"/>
       <c r="C46" s="5" t="s">
@@ -1674,7 +1679,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="47" spans="1:20" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="47" spans="1:20" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A47" s="17"/>
       <c r="B47" s="26"/>
       <c r="C47" s="5" t="s">
@@ -1689,7 +1694,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="48" spans="1:20" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="48" spans="1:20" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A48" s="17"/>
       <c r="B48" s="26"/>
       <c r="C48" s="5" t="s">
@@ -1704,7 +1709,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="49" spans="1:21" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="49" spans="1:21" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A49" s="17"/>
       <c r="B49" s="26"/>
       <c r="C49" s="5" t="s">
@@ -1719,7 +1724,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="50" spans="1:21" ht="159.5" x14ac:dyDescent="0.35">
+    <row r="50" spans="1:21" ht="158.4" x14ac:dyDescent="0.3">
       <c r="A50" s="19">
         <v>2</v>
       </c>
@@ -1740,7 +1745,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="51" spans="1:21" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="51" spans="1:21" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A51" s="26"/>
       <c r="B51" s="26"/>
       <c r="C51" s="5" t="s">
@@ -1757,7 +1762,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="52" spans="1:21" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="52" spans="1:21" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A52" s="19">
         <v>3</v>
       </c>
@@ -1776,7 +1781,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="53" spans="1:21" x14ac:dyDescent="0.35">
+    <row r="53" spans="1:21" x14ac:dyDescent="0.3">
       <c r="B53" s="5"/>
       <c r="C53" s="28" t="s">
         <v>18</v>
@@ -1792,7 +1797,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="54" spans="1:21" ht="58" x14ac:dyDescent="0.35">
+    <row r="54" spans="1:21" ht="57.6" x14ac:dyDescent="0.3">
       <c r="A54" s="19">
         <f>A52+1</f>
         <v>4</v>
@@ -1814,7 +1819,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="55" spans="1:21" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="55" spans="1:21" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A55" s="19">
         <f>A54+1</f>
         <v>5</v>
@@ -1834,7 +1839,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="56" spans="1:21" ht="29" x14ac:dyDescent="0.35">
+    <row r="56" spans="1:21" ht="28.8" x14ac:dyDescent="0.3">
       <c r="B56" s="5"/>
       <c r="C56" s="5" t="s">
         <v>24</v>
@@ -1848,7 +1853,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="57" spans="1:21" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="57" spans="1:21" ht="43.2" x14ac:dyDescent="0.3">
       <c r="B57" s="5"/>
       <c r="C57" s="5" t="s">
         <v>34</v>
@@ -1862,7 +1867,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="58" spans="1:21" ht="29" x14ac:dyDescent="0.35">
+    <row r="58" spans="1:21" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A58" s="19">
         <v>7</v>
       </c>
@@ -1880,7 +1885,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="59" spans="1:21" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="59" spans="1:21" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A59" s="5"/>
       <c r="B59" s="29" t="s">
         <v>36</v>
@@ -1891,7 +1896,7 @@
         <v>1.4285714285714286</v>
       </c>
     </row>
-    <row r="60" spans="1:21" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="60" spans="1:21" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A60" s="5"/>
       <c r="B60" s="29" t="s">
         <v>37</v>
@@ -1899,7 +1904,7 @@
       <c r="C60" s="5"/>
       <c r="F60" s="10">
         <f>F59+F39</f>
-        <v>3.3679653679653683</v>
+        <v>3.4285714285714288</v>
       </c>
       <c r="G60" s="10"/>
       <c r="H60" s="10"/>
@@ -1917,7 +1922,7 @@
       <c r="T60" s="10"/>
       <c r="U60" s="10"/>
     </row>
-    <row r="61" spans="1:21" x14ac:dyDescent="0.35">
+    <row r="61" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A61" s="5"/>
       <c r="B61" s="5"/>
       <c r="C61" s="5"/>
@@ -1962,22 +1967,22 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{578BE0C3-5829-4AF5-884F-BE3999CA7C49}">
   <dimension ref="A1:A3"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="12" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
         <v>8</v>
       </c>
     </row>
-    <row r="2" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>6</v>
       </c>
     </row>
-    <row r="3" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>7</v>
       </c>

</xml_diff>